<commit_message>
About page migration: fix chrome, sections, alignment, typography
- styles.css: scope content typography to match source (Oswald Bold headings
  in #20242d; section h2 32px, column h3 24px, timeline h4 20px, body 16px)
- transformers/hoegemeyer-cleanup.js: strip global header/footer experience
  fragments, breadcrumb, and TrustArc cookie-consent band (not page content)
- transformers/hoegemeyer-sections.js: split content into EDS sections and mark
  default-content groups text-center to match the live alignment
- import-about-page.js: drop fragment parser, wire sections transformer
- parsers/carousel.js: dedupe single-slide gallery
- page-templates.json: remove fragment mapping

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-page.report.xlsx
+++ b/tools/importer/reports/import-about-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>about.report.json</t>
   </si>
   <si>
-    <t>["teaser","carousel","columns","columns","columns","columns","columns","columns","columns","fragment","fragment"]</t>
+    <t>["teaser","carousel","columns","columns","columns","columns","columns","columns","columns"]</t>
   </si>
   <si>
     <t>about</t>
@@ -52,7 +52,7 @@
     <t>about-page</t>
   </si>
   <si>
-    <t>2026-08-19T05:48:08.201Z</t>
+    <t>2026-08-19T08:26:29.394Z</t>
   </si>
   <si>
     <t>About | Hoegemeyer Hybrids</t>

</xml_diff>

<commit_message>
About page: migrate breadcrumb block
- parsers/breadcrumb.js: convert source cmp-breadcrumb trail to the breadcrumb
  block (one crumb per row; link for navigable, plain text for current)
- transformers/hoegemeyer-cleanup.js: stop stripping .social-share (it hosts
  the breadcrumb); header/footer chrome and cookie band still removed
- import-about-page.js + page-templates.json: wire in the breadcrumb block

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-page.report.xlsx
+++ b/tools/importer/reports/import-about-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>about.report.json</t>
   </si>
   <si>
-    <t>["teaser","carousel","columns","columns","columns","columns","columns","columns","columns"]</t>
+    <t>["breadcrumb","teaser","carousel","columns","columns","columns","columns","columns","columns","columns"]</t>
   </si>
   <si>
     <t>about</t>
@@ -52,7 +52,7 @@
     <t>about-page</t>
   </si>
   <si>
-    <t>2026-08-19T08:26:29.394Z</t>
+    <t>2026-08-19T08:38:38.836Z</t>
   </si>
   <si>
     <t>About | Hoegemeyer Hybrids</t>

</xml_diff>